<commit_message>
chore: update IPO tracker data
</commit_message>
<xml_diff>
--- a/data/mainboard_ipos.xlsx
+++ b/data/mainboard_ipos.xlsx
@@ -2677,7 +2677,7 @@
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>2026-09-12 23:14:55</t>
+          <t>2026-09-13 13:49:32</t>
         </is>
       </c>
     </row>
@@ -2761,7 +2761,7 @@
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>2026-09-12 23:14:55</t>
+          <t>2026-09-13 13:49:32</t>
         </is>
       </c>
     </row>
@@ -2897,7 +2897,7 @@
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>2026-09-12 23:14:55</t>
+          <t>2026-09-13 13:49:32</t>
         </is>
       </c>
     </row>
@@ -3101,7 +3101,7 @@
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>2026-09-12 23:14:55</t>
+          <t>2026-09-13 13:49:32</t>
         </is>
       </c>
     </row>
@@ -3169,7 +3169,7 @@
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>2026-09-12 23:14:55</t>
+          <t>2026-09-13 13:49:32</t>
         </is>
       </c>
     </row>
@@ -3509,7 +3509,7 @@
       </c>
       <c r="R39" t="inlineStr">
         <is>
-          <t>2026-09-12 23:14:55</t>
+          <t>2026-09-13 13:49:32</t>
         </is>
       </c>
     </row>
@@ -3577,7 +3577,7 @@
       </c>
       <c r="R40" t="inlineStr">
         <is>
-          <t>2026-09-12 23:14:55</t>
+          <t>2026-09-13 13:49:32</t>
         </is>
       </c>
     </row>
@@ -3641,7 +3641,7 @@
       </c>
       <c r="R41" t="inlineStr">
         <is>
-          <t>2026-09-12 23:14:55</t>
+          <t>2026-09-13 13:49:32</t>
         </is>
       </c>
     </row>
@@ -3705,7 +3705,7 @@
       </c>
       <c r="R42" t="inlineStr">
         <is>
-          <t>2026-09-12 23:14:55</t>
+          <t>2026-09-13 13:49:32</t>
         </is>
       </c>
     </row>
@@ -3769,7 +3769,7 @@
       </c>
       <c r="R43" t="inlineStr">
         <is>
-          <t>2026-09-12 23:14:55</t>
+          <t>2026-09-13 13:49:32</t>
         </is>
       </c>
     </row>
@@ -3833,7 +3833,7 @@
       </c>
       <c r="R44" t="inlineStr">
         <is>
-          <t>2026-09-12 23:14:55</t>
+          <t>2026-09-13 13:49:32</t>
         </is>
       </c>
     </row>
@@ -3897,7 +3897,7 @@
       </c>
       <c r="R45" t="inlineStr">
         <is>
-          <t>2026-09-12 23:14:55</t>
+          <t>2026-09-13 13:49:32</t>
         </is>
       </c>
     </row>

</xml_diff>